<commit_message>
doc: update daily notes and workfiles - add labeled-project and Functional Block exercises - update io-mapping to include non-duplicate names for sensor/output
</commit_message>
<xml_diff>
--- a/plc/plc-io-map.xlsx
+++ b/plc/plc-io-map.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_최예현\PLC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_최예현\intel26\plc\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12255" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12255"/>
   </bookViews>
   <sheets>
     <sheet name="Data Parameter" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="111">
   <si>
     <t>X0</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -124,14 +124,6 @@
   </si>
   <si>
     <t>공급_전</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>드릴_상</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>드릴_하</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -400,6 +392,38 @@
   <si>
     <t>CPU -&gt; D/A
 CH1 allow/deny (1 / 0)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>공급_후_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>공급_전_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>드릴_상_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>드릴_하_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>송출_후_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>송출_전_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>배출_후_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>배출_전_완</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1095,19 +1119,19 @@
         <v>10</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>14</v>
       </c>
       <c r="J3" s="38" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K3" s="39"/>
     </row>
@@ -1116,13 +1140,13 @@
         <v>0</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>27</v>
+        <v>103</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>12</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>15</v>
@@ -1131,7 +1155,7 @@
         <v>28</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1139,13 +1163,13 @@
         <v>1</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>16</v>
@@ -1154,7 +1178,7 @@
         <v>27</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1162,22 +1186,22 @@
         <v>2</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1185,20 +1209,20 @@
         <v>3</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>30</v>
+        <v>106</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H7" s="5"/>
       <c r="I7" s="1" t="s">
         <v>18</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1206,20 +1230,20 @@
         <v>4</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>31</v>
+        <v>107</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H8" s="5"/>
       <c r="I8" s="1" t="s">
         <v>19</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1227,20 +1251,20 @@
         <v>5</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>32</v>
+        <v>108</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="H9" s="5"/>
       <c r="I9" s="1" t="s">
         <v>20</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1248,20 +1272,20 @@
         <v>6</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>33</v>
+        <v>109</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H10" s="5"/>
       <c r="I10" s="1" t="s">
         <v>21</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1269,17 +1293,17 @@
         <v>7</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>34</v>
+        <v>110</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="1" t="s">
         <v>22</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="K11" s="5"/>
     </row>
@@ -1288,19 +1312,19 @@
         <v>8</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>23</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="K12" s="5"/>
     </row>
@@ -1309,7 +1333,7 @@
         <v>9</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="5"/>
@@ -1317,24 +1341,24 @@
         <v>24</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="K13" s="6"/>
     </row>
     <row r="14" spans="5:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E14" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="K14" s="6"/>
     </row>
@@ -1344,10 +1368,10 @@
       <c r="G15" s="5"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="K15" s="6"/>
     </row>
@@ -1362,18 +1386,18 @@
     </row>
     <row r="17" spans="5:11" ht="33" x14ac:dyDescent="0.3">
       <c r="E17" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F17" s="32" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G17" s="5"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="J17" s="32" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="K17" s="6"/>
     </row>
@@ -1450,20 +1474,20 @@
   <sheetData>
     <row r="1" spans="2:26" x14ac:dyDescent="0.3">
       <c r="M1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="2:26" x14ac:dyDescent="0.3">
       <c r="C2" s="31" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="M2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="2:26" x14ac:dyDescent="0.3">
       <c r="C3" s="31" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="2:26" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -1508,39 +1532,39 @@
         <v>1</v>
       </c>
       <c r="X5" s="30" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="2:26" x14ac:dyDescent="0.3">
       <c r="E6" s="27" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F6" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="H6" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="I6" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="G6" s="28" t="s">
-        <v>51</v>
-      </c>
-      <c r="H6" s="29" t="s">
-        <v>68</v>
-      </c>
-      <c r="I6" s="27" t="s">
-        <v>54</v>
-      </c>
       <c r="J6" s="28" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K6" s="28" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="L6" s="29" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="M6" s="27" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="N6" s="28" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="O6" s="28" t="s">
         <v>27</v>
@@ -1552,15 +1576,15 @@
         <v>2</v>
       </c>
       <c r="X6" s="30" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="2:26" x14ac:dyDescent="0.3">
       <c r="E7" s="27" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F7" s="28" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G7" s="28" t="s">
         <v>24</v>
@@ -1587,7 +1611,7 @@
         <v>17</v>
       </c>
       <c r="O7" s="28" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="P7" s="29" t="s">
         <v>15</v>
@@ -1596,15 +1620,15 @@
         <v>3</v>
       </c>
       <c r="X7" s="30" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
@@ -1662,15 +1686,15 @@
         <v>4</v>
       </c>
       <c r="X8" s="30" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="2:26" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E9" s="15">
         <v>0</v>
@@ -1728,7 +1752,7 @@
         <v>5</v>
       </c>
       <c r="X9" s="30" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="2:26" x14ac:dyDescent="0.3">
@@ -1736,7 +1760,7 @@
         <v>6</v>
       </c>
       <c r="X10" s="30" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="2:26" x14ac:dyDescent="0.3">
@@ -1744,12 +1768,12 @@
         <v>7</v>
       </c>
       <c r="X11" s="30" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="2:26" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -1780,7 +1804,7 @@
         <v>8</v>
       </c>
       <c r="X12" s="30" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="Z12" t="str">
         <f>CONCATENATE("MOV H",U12," K3Y20")</f>
@@ -1789,7 +1813,7 @@
     </row>
     <row r="13" spans="2:26" x14ac:dyDescent="0.3">
       <c r="D13" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -1820,7 +1844,7 @@
         <v>9</v>
       </c>
       <c r="X13" s="30" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="Z13" t="str">
         <f t="shared" ref="Z13:Z20" si="4">CONCATENATE("MOV H",U13," K3Y20")</f>
@@ -1829,7 +1853,7 @@
     </row>
     <row r="14" spans="2:26" x14ac:dyDescent="0.3">
       <c r="D14" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="M14">
         <v>1</v>
@@ -1857,7 +1881,7 @@
         <v>10</v>
       </c>
       <c r="X14" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="Z14" t="str">
         <f t="shared" si="4"/>
@@ -1866,7 +1890,7 @@
     </row>
     <row r="15" spans="2:26" x14ac:dyDescent="0.3">
       <c r="D15" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -1894,7 +1918,7 @@
         <v>11</v>
       </c>
       <c r="X15" s="7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="Z15" t="str">
         <f t="shared" si="4"/>
@@ -1903,7 +1927,7 @@
     </row>
     <row r="16" spans="2:26" x14ac:dyDescent="0.3">
       <c r="D16" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="L16">
         <v>1</v>
@@ -1931,7 +1955,7 @@
         <v>12</v>
       </c>
       <c r="X16" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="Z16" t="str">
         <f t="shared" si="4"/>
@@ -1940,7 +1964,7 @@
     </row>
     <row r="17" spans="4:26" x14ac:dyDescent="0.3">
       <c r="D17" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="N17">
         <v>0</v>
@@ -1965,7 +1989,7 @@
         <v>13</v>
       </c>
       <c r="X17" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="Z17" t="str">
         <f t="shared" si="4"/>
@@ -1974,7 +1998,7 @@
     </row>
     <row r="18" spans="4:26" x14ac:dyDescent="0.3">
       <c r="D18" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="K18">
         <v>1</v>
@@ -1999,7 +2023,7 @@
         <v>14</v>
       </c>
       <c r="X18" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="Z18" t="str">
         <f t="shared" si="4"/>
@@ -2008,7 +2032,7 @@
     </row>
     <row r="19" spans="4:26" x14ac:dyDescent="0.3">
       <c r="D19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J19">
         <v>1</v>
@@ -2033,7 +2057,7 @@
         <v>15</v>
       </c>
       <c r="X19" s="7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="Z19" t="str">
         <f t="shared" si="4"/>
@@ -2042,7 +2066,7 @@
     </row>
     <row r="20" spans="4:26" x14ac:dyDescent="0.3">
       <c r="D20" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="R20" s="26" t="str">
         <f t="shared" ref="R20" si="5">IFERROR(VLOOKUP(E20*E$5+F20*F$5+G20*G$5+H20*H$5,$W$5:$X$19,2),"0")</f>
@@ -2079,20 +2103,20 @@
   <sheetData>
     <row r="1" spans="2:29" x14ac:dyDescent="0.3">
       <c r="Q1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="2:29" x14ac:dyDescent="0.3">
       <c r="C2" s="31" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="Q2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="2:29" x14ac:dyDescent="0.3">
       <c r="C3" s="31" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="2:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -2149,7 +2173,7 @@
         <v>1</v>
       </c>
       <c r="AC5" s="30" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="2:29" x14ac:dyDescent="0.3">
@@ -2173,7 +2197,7 @@
         <v>2</v>
       </c>
       <c r="AC6" s="30" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="2:29" x14ac:dyDescent="0.3">
@@ -2197,15 +2221,15 @@
         <v>3</v>
       </c>
       <c r="AC7" s="30" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
@@ -2279,15 +2303,15 @@
         <v>4</v>
       </c>
       <c r="AC8" s="30" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="2:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E9" s="15">
         <v>0</v>
@@ -2361,7 +2385,7 @@
         <v>5</v>
       </c>
       <c r="AC9" s="30" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="2:29" x14ac:dyDescent="0.3">
@@ -2369,7 +2393,7 @@
         <v>6</v>
       </c>
       <c r="AC10" s="30" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="2:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2377,7 +2401,7 @@
         <v>7</v>
       </c>
       <c r="AC11" s="30" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="2:29" x14ac:dyDescent="0.3">
@@ -2453,7 +2477,7 @@
         <v>8</v>
       </c>
       <c r="AC12" s="30" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="2:29" x14ac:dyDescent="0.3">
@@ -2497,7 +2521,7 @@
         <v>9</v>
       </c>
       <c r="AC13" s="30" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="2:29" x14ac:dyDescent="0.3">
@@ -2528,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="AC14" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="2:29" x14ac:dyDescent="0.3">
@@ -2559,7 +2583,7 @@
         <v>11</v>
       </c>
       <c r="AC15" s="7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="2:29" x14ac:dyDescent="0.3">
@@ -2590,7 +2614,7 @@
         <v>12</v>
       </c>
       <c r="AC16" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="5:29" x14ac:dyDescent="0.3">
@@ -2621,7 +2645,7 @@
         <v>13</v>
       </c>
       <c r="AC17" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="18" spans="5:29" x14ac:dyDescent="0.3">
@@ -2652,7 +2676,7 @@
         <v>14</v>
       </c>
       <c r="AC18" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="5:29" x14ac:dyDescent="0.3">
@@ -2683,7 +2707,7 @@
         <v>15</v>
       </c>
       <c r="AC19" s="7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="5:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
doc: update daily notes and workfiles (#2)
* doc: update readme for repo and subsections
* doc: change wording of exam
* doc: update daily notes and workfiles
</commit_message>
<xml_diff>
--- a/plc/plc-io-map.xlsx
+++ b/plc/plc-io-map.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_최예현\PLC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_최예현\intel26\plc\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12255" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12255"/>
   </bookViews>
   <sheets>
     <sheet name="Data Parameter" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="111">
   <si>
     <t>X0</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -124,14 +124,6 @@
   </si>
   <si>
     <t>공급_전</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>드릴_상</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>드릴_하</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -400,6 +392,38 @@
   <si>
     <t>CPU -&gt; D/A
 CH1 allow/deny (1 / 0)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>공급_후_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>공급_전_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>드릴_상_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>드릴_하_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>송출_후_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>송출_전_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>배출_후_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>배출_전_완</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1095,19 +1119,19 @@
         <v>10</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>14</v>
       </c>
       <c r="J3" s="38" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K3" s="39"/>
     </row>
@@ -1116,13 +1140,13 @@
         <v>0</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>27</v>
+        <v>103</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>12</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>15</v>
@@ -1131,7 +1155,7 @@
         <v>28</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1139,13 +1163,13 @@
         <v>1</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>16</v>
@@ -1154,7 +1178,7 @@
         <v>27</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1162,22 +1186,22 @@
         <v>2</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1185,20 +1209,20 @@
         <v>3</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>30</v>
+        <v>106</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H7" s="5"/>
       <c r="I7" s="1" t="s">
         <v>18</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1206,20 +1230,20 @@
         <v>4</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>31</v>
+        <v>107</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H8" s="5"/>
       <c r="I8" s="1" t="s">
         <v>19</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1227,20 +1251,20 @@
         <v>5</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>32</v>
+        <v>108</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="H9" s="5"/>
       <c r="I9" s="1" t="s">
         <v>20</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1248,20 +1272,20 @@
         <v>6</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>33</v>
+        <v>109</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H10" s="5"/>
       <c r="I10" s="1" t="s">
         <v>21</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1269,17 +1293,17 @@
         <v>7</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>34</v>
+        <v>110</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="1" t="s">
         <v>22</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="K11" s="5"/>
     </row>
@@ -1288,19 +1312,19 @@
         <v>8</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>23</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="K12" s="5"/>
     </row>
@@ -1309,7 +1333,7 @@
         <v>9</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="5"/>
@@ -1317,24 +1341,24 @@
         <v>24</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="K13" s="6"/>
     </row>
     <row r="14" spans="5:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E14" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="K14" s="6"/>
     </row>
@@ -1344,10 +1368,10 @@
       <c r="G15" s="5"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="K15" s="6"/>
     </row>
@@ -1362,18 +1386,18 @@
     </row>
     <row r="17" spans="5:11" ht="33" x14ac:dyDescent="0.3">
       <c r="E17" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F17" s="32" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G17" s="5"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="J17" s="32" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="K17" s="6"/>
     </row>
@@ -1450,20 +1474,20 @@
   <sheetData>
     <row r="1" spans="2:26" x14ac:dyDescent="0.3">
       <c r="M1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="2:26" x14ac:dyDescent="0.3">
       <c r="C2" s="31" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="M2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="2:26" x14ac:dyDescent="0.3">
       <c r="C3" s="31" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="2:26" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -1508,39 +1532,39 @@
         <v>1</v>
       </c>
       <c r="X5" s="30" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="2:26" x14ac:dyDescent="0.3">
       <c r="E6" s="27" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F6" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="H6" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="I6" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="G6" s="28" t="s">
-        <v>51</v>
-      </c>
-      <c r="H6" s="29" t="s">
-        <v>68</v>
-      </c>
-      <c r="I6" s="27" t="s">
-        <v>54</v>
-      </c>
       <c r="J6" s="28" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K6" s="28" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="L6" s="29" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="M6" s="27" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="N6" s="28" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="O6" s="28" t="s">
         <v>27</v>
@@ -1552,15 +1576,15 @@
         <v>2</v>
       </c>
       <c r="X6" s="30" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="2:26" x14ac:dyDescent="0.3">
       <c r="E7" s="27" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F7" s="28" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G7" s="28" t="s">
         <v>24</v>
@@ -1587,7 +1611,7 @@
         <v>17</v>
       </c>
       <c r="O7" s="28" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="P7" s="29" t="s">
         <v>15</v>
@@ -1596,15 +1620,15 @@
         <v>3</v>
       </c>
       <c r="X7" s="30" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
@@ -1662,15 +1686,15 @@
         <v>4</v>
       </c>
       <c r="X8" s="30" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="2:26" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E9" s="15">
         <v>0</v>
@@ -1728,7 +1752,7 @@
         <v>5</v>
       </c>
       <c r="X9" s="30" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="2:26" x14ac:dyDescent="0.3">
@@ -1736,7 +1760,7 @@
         <v>6</v>
       </c>
       <c r="X10" s="30" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="2:26" x14ac:dyDescent="0.3">
@@ -1744,12 +1768,12 @@
         <v>7</v>
       </c>
       <c r="X11" s="30" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="2:26" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -1780,7 +1804,7 @@
         <v>8</v>
       </c>
       <c r="X12" s="30" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="Z12" t="str">
         <f>CONCATENATE("MOV H",U12," K3Y20")</f>
@@ -1789,7 +1813,7 @@
     </row>
     <row r="13" spans="2:26" x14ac:dyDescent="0.3">
       <c r="D13" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -1820,7 +1844,7 @@
         <v>9</v>
       </c>
       <c r="X13" s="30" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="Z13" t="str">
         <f t="shared" ref="Z13:Z20" si="4">CONCATENATE("MOV H",U13," K3Y20")</f>
@@ -1829,7 +1853,7 @@
     </row>
     <row r="14" spans="2:26" x14ac:dyDescent="0.3">
       <c r="D14" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="M14">
         <v>1</v>
@@ -1857,7 +1881,7 @@
         <v>10</v>
       </c>
       <c r="X14" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="Z14" t="str">
         <f t="shared" si="4"/>
@@ -1866,7 +1890,7 @@
     </row>
     <row r="15" spans="2:26" x14ac:dyDescent="0.3">
       <c r="D15" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -1894,7 +1918,7 @@
         <v>11</v>
       </c>
       <c r="X15" s="7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="Z15" t="str">
         <f t="shared" si="4"/>
@@ -1903,7 +1927,7 @@
     </row>
     <row r="16" spans="2:26" x14ac:dyDescent="0.3">
       <c r="D16" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="L16">
         <v>1</v>
@@ -1931,7 +1955,7 @@
         <v>12</v>
       </c>
       <c r="X16" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="Z16" t="str">
         <f t="shared" si="4"/>
@@ -1940,7 +1964,7 @@
     </row>
     <row r="17" spans="4:26" x14ac:dyDescent="0.3">
       <c r="D17" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="N17">
         <v>0</v>
@@ -1965,7 +1989,7 @@
         <v>13</v>
       </c>
       <c r="X17" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="Z17" t="str">
         <f t="shared" si="4"/>
@@ -1974,7 +1998,7 @@
     </row>
     <row r="18" spans="4:26" x14ac:dyDescent="0.3">
       <c r="D18" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="K18">
         <v>1</v>
@@ -1999,7 +2023,7 @@
         <v>14</v>
       </c>
       <c r="X18" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="Z18" t="str">
         <f t="shared" si="4"/>
@@ -2008,7 +2032,7 @@
     </row>
     <row r="19" spans="4:26" x14ac:dyDescent="0.3">
       <c r="D19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J19">
         <v>1</v>
@@ -2033,7 +2057,7 @@
         <v>15</v>
       </c>
       <c r="X19" s="7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="Z19" t="str">
         <f t="shared" si="4"/>
@@ -2042,7 +2066,7 @@
     </row>
     <row r="20" spans="4:26" x14ac:dyDescent="0.3">
       <c r="D20" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="R20" s="26" t="str">
         <f t="shared" ref="R20" si="5">IFERROR(VLOOKUP(E20*E$5+F20*F$5+G20*G$5+H20*H$5,$W$5:$X$19,2),"0")</f>
@@ -2079,20 +2103,20 @@
   <sheetData>
     <row r="1" spans="2:29" x14ac:dyDescent="0.3">
       <c r="Q1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="2:29" x14ac:dyDescent="0.3">
       <c r="C2" s="31" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="Q2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="2:29" x14ac:dyDescent="0.3">
       <c r="C3" s="31" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="2:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -2149,7 +2173,7 @@
         <v>1</v>
       </c>
       <c r="AC5" s="30" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="2:29" x14ac:dyDescent="0.3">
@@ -2173,7 +2197,7 @@
         <v>2</v>
       </c>
       <c r="AC6" s="30" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="2:29" x14ac:dyDescent="0.3">
@@ -2197,15 +2221,15 @@
         <v>3</v>
       </c>
       <c r="AC7" s="30" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
@@ -2279,15 +2303,15 @@
         <v>4</v>
       </c>
       <c r="AC8" s="30" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="2:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E9" s="15">
         <v>0</v>
@@ -2361,7 +2385,7 @@
         <v>5</v>
       </c>
       <c r="AC9" s="30" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="2:29" x14ac:dyDescent="0.3">
@@ -2369,7 +2393,7 @@
         <v>6</v>
       </c>
       <c r="AC10" s="30" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="2:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2377,7 +2401,7 @@
         <v>7</v>
       </c>
       <c r="AC11" s="30" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="2:29" x14ac:dyDescent="0.3">
@@ -2453,7 +2477,7 @@
         <v>8</v>
       </c>
       <c r="AC12" s="30" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="2:29" x14ac:dyDescent="0.3">
@@ -2497,7 +2521,7 @@
         <v>9</v>
       </c>
       <c r="AC13" s="30" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="2:29" x14ac:dyDescent="0.3">
@@ -2528,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="AC14" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="2:29" x14ac:dyDescent="0.3">
@@ -2559,7 +2583,7 @@
         <v>11</v>
       </c>
       <c r="AC15" s="7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="2:29" x14ac:dyDescent="0.3">
@@ -2590,7 +2614,7 @@
         <v>12</v>
       </c>
       <c r="AC16" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="5:29" x14ac:dyDescent="0.3">
@@ -2621,7 +2645,7 @@
         <v>13</v>
       </c>
       <c r="AC17" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="18" spans="5:29" x14ac:dyDescent="0.3">
@@ -2652,7 +2676,7 @@
         <v>14</v>
       </c>
       <c r="AC18" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="5:29" x14ac:dyDescent="0.3">
@@ -2683,7 +2707,7 @@
         <v>15</v>
       </c>
       <c r="AC19" s="7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="5:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
docs: add plc practice projects and notes
- remove repeat notes txt for 0716
- add 0722 notes
- add ethernet, and more practice exam projects
</commit_message>
<xml_diff>
--- a/plc/plc-io-map.xlsx
+++ b/plc/plc-io-map.xlsx
@@ -257,10 +257,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>드릴</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>가공모터</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -424,6 +420,10 @@
   </si>
   <si>
     <t>배출_전_완</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>가공</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -473,7 +473,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -519,6 +519,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -689,7 +695,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -809,6 +815,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1140,7 +1149,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>12</v>
@@ -1163,7 +1172,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>13</v>
@@ -1186,7 +1195,7 @@
         <v>2</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>44</v>
@@ -1209,7 +1218,7 @@
         <v>3</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>57</v>
@@ -1230,7 +1239,7 @@
         <v>4</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>58</v>
@@ -1251,7 +1260,7 @@
         <v>5</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>59</v>
@@ -1272,7 +1281,7 @@
         <v>6</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>60</v>
@@ -1293,7 +1302,7 @@
         <v>7</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>61</v>
@@ -1386,18 +1395,18 @@
     </row>
     <row r="17" spans="5:11" ht="33" x14ac:dyDescent="0.3">
       <c r="E17" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F17" s="32" t="s">
         <v>99</v>
-      </c>
-      <c r="F17" s="32" t="s">
-        <v>100</v>
       </c>
       <c r="G17" s="5"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="J17" s="32" t="s">
         <v>101</v>
-      </c>
-      <c r="J17" s="32" t="s">
-        <v>102</v>
       </c>
       <c r="K17" s="6"/>
     </row>
@@ -1474,20 +1483,20 @@
   <sheetData>
     <row r="1" spans="2:26" x14ac:dyDescent="0.3">
       <c r="M1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="2:26" x14ac:dyDescent="0.3">
       <c r="C2" s="31" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="2:26" x14ac:dyDescent="0.3">
       <c r="C3" s="31" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="2:26" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -1532,7 +1541,7 @@
         <v>1</v>
       </c>
       <c r="X5" s="30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="2:26" x14ac:dyDescent="0.3">
@@ -1546,7 +1555,7 @@
         <v>49</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I6" s="27" t="s">
         <v>52</v>
@@ -1564,7 +1573,7 @@
         <v>30</v>
       </c>
       <c r="N6" s="28" t="s">
-        <v>65</v>
+        <v>110</v>
       </c>
       <c r="O6" s="28" t="s">
         <v>27</v>
@@ -1576,7 +1585,7 @@
         <v>2</v>
       </c>
       <c r="X6" s="30" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="2:26" x14ac:dyDescent="0.3">
@@ -1620,15 +1629,15 @@
         <v>3</v>
       </c>
       <c r="X7" s="30" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
@@ -1686,15 +1695,15 @@
         <v>4</v>
       </c>
       <c r="X8" s="30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="2:26" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E9" s="15">
         <v>0</v>
@@ -1752,7 +1761,7 @@
         <v>5</v>
       </c>
       <c r="X9" s="30" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="2:26" x14ac:dyDescent="0.3">
@@ -1760,7 +1769,7 @@
         <v>6</v>
       </c>
       <c r="X10" s="30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="2:26" x14ac:dyDescent="0.3">
@@ -1768,25 +1777,30 @@
         <v>7</v>
       </c>
       <c r="X11" s="30" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="D12" t="s">
-        <v>86</v>
-      </c>
-      <c r="E12">
-        <v>1</v>
-      </c>
-      <c r="N12">
-        <v>0</v>
-      </c>
-      <c r="P12">
+      <c r="D12" s="40" t="s">
+        <v>85</v>
+      </c>
+      <c r="E12" s="40"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="40"/>
+      <c r="H12" s="40"/>
+      <c r="I12" s="40"/>
+      <c r="J12" s="40"/>
+      <c r="K12" s="40"/>
+      <c r="L12" s="40"/>
+      <c r="M12" s="40"/>
+      <c r="N12" s="40"/>
+      <c r="O12" s="40"/>
+      <c r="P12" s="40">
         <v>1</v>
       </c>
       <c r="R12" s="26" t="str">
         <f t="shared" ref="R12:R19" si="0">IFERROR(VLOOKUP(E12*E$5+F12*F$5+G12*G$5+H12*H$5,$W$5:$X$19,2),"0")</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S12" s="26" t="str">
         <f t="shared" ref="S12:S19" si="1">IFERROR(VLOOKUP(I12*I$5+J12*J$5+K12*K$5+L12*L$5,$W$5:$X$19,2),"0")</f>
@@ -1798,35 +1812,32 @@
       </c>
       <c r="U12" t="str">
         <f t="shared" ref="U12:U19" si="3">CONCATENATE(R12,S12,T12)</f>
-        <v>801</v>
+        <v>001</v>
       </c>
       <c r="W12" s="7">
         <v>8</v>
       </c>
       <c r="X12" s="30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="Z12" t="str">
         <f>CONCATENATE("MOV H",U12," K3Y20")</f>
-        <v>MOV H801 K3Y20</v>
+        <v>MOV H001 K3Y20</v>
       </c>
     </row>
     <row r="13" spans="2:26" x14ac:dyDescent="0.3">
       <c r="D13" t="s">
-        <v>87</v>
-      </c>
-      <c r="E13">
-        <v>1</v>
-      </c>
-      <c r="N13">
-        <v>1</v>
-      </c>
-      <c r="O13">
-        <v>1</v>
+        <v>86</v>
+      </c>
+      <c r="M13">
+        <v>1</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
       </c>
       <c r="R13" s="26" t="str">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S13" s="26" t="str">
         <f t="shared" si="1"/>
@@ -1834,36 +1845,48 @@
       </c>
       <c r="T13" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U13" t="str">
         <f t="shared" si="3"/>
-        <v>806</v>
+        <v>008</v>
       </c>
       <c r="W13" s="7">
         <v>9</v>
       </c>
       <c r="X13" s="30" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="Z13" t="str">
         <f t="shared" ref="Z13:Z20" si="4">CONCATENATE("MOV H",U13," K3Y20")</f>
-        <v>MOV H806 K3Y20</v>
+        <v>MOV H008 K3Y20</v>
       </c>
     </row>
     <row r="14" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="D14" t="s">
-        <v>88</v>
-      </c>
-      <c r="M14">
-        <v>1</v>
-      </c>
-      <c r="N14">
-        <v>1</v>
+      <c r="D14" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="E14" s="40"/>
+      <c r="F14" s="40">
+        <v>1</v>
+      </c>
+      <c r="G14" s="40"/>
+      <c r="H14" s="40"/>
+      <c r="I14" s="40"/>
+      <c r="J14" s="40"/>
+      <c r="K14" s="40"/>
+      <c r="L14" s="40"/>
+      <c r="M14" s="40"/>
+      <c r="N14" s="40">
+        <v>1</v>
+      </c>
+      <c r="O14" s="40"/>
+      <c r="P14" s="40">
+        <v>0</v>
       </c>
       <c r="R14" s="26" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="S14" s="26" t="str">
         <f t="shared" si="1"/>
@@ -1871,31 +1894,34 @@
       </c>
       <c r="T14" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>C</v>
+        <v>4</v>
       </c>
       <c r="U14" t="str">
         <f t="shared" si="3"/>
-        <v>00C</v>
+        <v>404</v>
       </c>
       <c r="W14" s="7">
         <v>10</v>
       </c>
       <c r="X14" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="Z14" t="str">
         <f t="shared" si="4"/>
-        <v>MOV H00C K3Y20</v>
+        <v>MOV H404 K3Y20</v>
       </c>
     </row>
     <row r="15" spans="2:26" x14ac:dyDescent="0.3">
       <c r="D15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F15">
         <v>1</v>
       </c>
       <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
         <v>1</v>
       </c>
       <c r="R15" s="26" t="str">
@@ -1908,70 +1934,80 @@
       </c>
       <c r="T15" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U15" t="str">
         <f t="shared" si="3"/>
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="W15" s="7">
         <v>11</v>
       </c>
       <c r="X15" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Z15" t="str">
         <f t="shared" si="4"/>
-        <v>MOV H404 K3Y20</v>
+        <v>MOV H402 K3Y20</v>
       </c>
     </row>
     <row r="16" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="D16" t="s">
-        <v>90</v>
-      </c>
-      <c r="L16">
-        <v>1</v>
-      </c>
-      <c r="N16">
-        <v>1</v>
-      </c>
+      <c r="D16" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="E16" s="40"/>
+      <c r="F16" s="40">
+        <v>0</v>
+      </c>
+      <c r="G16" s="40"/>
+      <c r="H16" s="40"/>
+      <c r="I16" s="40"/>
+      <c r="J16" s="40"/>
+      <c r="K16" s="40">
+        <v>1</v>
+      </c>
+      <c r="L16" s="40"/>
+      <c r="M16" s="40"/>
+      <c r="N16" s="40"/>
+      <c r="O16" s="40"/>
+      <c r="P16" s="40"/>
       <c r="R16" s="26" t="str">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="S16" s="26" t="str">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T16" s="26" t="str">
         <f t="shared" si="2"/>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="U16" t="str">
         <f t="shared" si="3"/>
-        <v>014</v>
+        <v>020</v>
       </c>
       <c r="W16" s="7">
         <v>12</v>
       </c>
       <c r="X16" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Z16" t="str">
         <f t="shared" si="4"/>
-        <v>MOV H014 K3Y20</v>
+        <v>MOV H020 K3Y20</v>
       </c>
     </row>
     <row r="17" spans="4:26" x14ac:dyDescent="0.3">
       <c r="D17" t="s">
-        <v>91</v>
-      </c>
-      <c r="N17">
-        <v>0</v>
+        <v>90</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
       </c>
       <c r="R17" s="26" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="S17" s="26" t="str">
         <f t="shared" si="1"/>
@@ -1983,33 +2019,46 @@
       </c>
       <c r="U17" t="str">
         <f t="shared" si="3"/>
-        <v>000</v>
+        <v>800</v>
       </c>
       <c r="W17" s="7">
         <v>13</v>
       </c>
       <c r="X17" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Z17" t="str">
         <f t="shared" si="4"/>
-        <v>MOV H000 K3Y20</v>
+        <v>MOV H800 K3Y20</v>
       </c>
     </row>
     <row r="18" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D18" t="s">
-        <v>92</v>
-      </c>
-      <c r="K18">
-        <v>1</v>
-      </c>
+      <c r="D18" s="40" t="s">
+        <v>91</v>
+      </c>
+      <c r="E18" s="40">
+        <v>0</v>
+      </c>
+      <c r="F18" s="40"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="40"/>
+      <c r="I18" s="40"/>
+      <c r="J18" s="40">
+        <v>1</v>
+      </c>
+      <c r="K18" s="40"/>
+      <c r="L18" s="40"/>
+      <c r="M18" s="40"/>
+      <c r="N18" s="40"/>
+      <c r="O18" s="40"/>
+      <c r="P18" s="40"/>
       <c r="R18" s="26" t="str">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="S18" s="26" t="str">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T18" s="26" t="str">
         <f t="shared" si="2"/>
@@ -2017,24 +2066,24 @@
       </c>
       <c r="U18" t="str">
         <f t="shared" si="3"/>
-        <v>020</v>
+        <v>040</v>
       </c>
       <c r="W18" s="7">
         <v>14</v>
       </c>
       <c r="X18" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="Z18" t="str">
         <f t="shared" si="4"/>
-        <v>MOV H020 K3Y20</v>
+        <v>MOV H040 K3Y20</v>
       </c>
     </row>
     <row r="19" spans="4:26" x14ac:dyDescent="0.3">
       <c r="D19" t="s">
-        <v>93</v>
-      </c>
-      <c r="J19">
+        <v>92</v>
+      </c>
+      <c r="L19">
         <v>1</v>
       </c>
       <c r="R19" s="26" t="str">
@@ -2043,7 +2092,7 @@
       </c>
       <c r="S19" s="26" t="str">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T19" s="26" t="str">
         <f t="shared" si="2"/>
@@ -2051,23 +2100,35 @@
       </c>
       <c r="U19" t="str">
         <f t="shared" si="3"/>
-        <v>040</v>
+        <v>010</v>
       </c>
       <c r="W19" s="7">
         <v>15</v>
       </c>
       <c r="X19" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Z19" t="str">
         <f t="shared" si="4"/>
-        <v>MOV H040 K3Y20</v>
+        <v>MOV H010 K3Y20</v>
       </c>
     </row>
     <row r="20" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D20" t="s">
-        <v>94</v>
-      </c>
+      <c r="D20" s="40" t="s">
+        <v>93</v>
+      </c>
+      <c r="E20" s="40"/>
+      <c r="F20" s="40"/>
+      <c r="G20" s="40"/>
+      <c r="H20" s="40"/>
+      <c r="I20" s="40"/>
+      <c r="J20" s="40"/>
+      <c r="K20" s="40"/>
+      <c r="L20" s="40"/>
+      <c r="M20" s="40"/>
+      <c r="N20" s="40"/>
+      <c r="O20" s="40"/>
+      <c r="P20" s="40"/>
       <c r="R20" s="26" t="str">
         <f t="shared" ref="R20" si="5">IFERROR(VLOOKUP(E20*E$5+F20*F$5+G20*G$5+H20*H$5,$W$5:$X$19,2),"0")</f>
         <v>0</v>
@@ -2103,20 +2164,20 @@
   <sheetData>
     <row r="1" spans="2:29" x14ac:dyDescent="0.3">
       <c r="Q1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="2:29" x14ac:dyDescent="0.3">
       <c r="C2" s="31" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="Q2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="2:29" x14ac:dyDescent="0.3">
       <c r="C3" s="31" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="2:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -2173,7 +2234,7 @@
         <v>1</v>
       </c>
       <c r="AC5" s="30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="2:29" x14ac:dyDescent="0.3">
@@ -2197,7 +2258,7 @@
         <v>2</v>
       </c>
       <c r="AC6" s="30" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="2:29" x14ac:dyDescent="0.3">
@@ -2221,15 +2282,15 @@
         <v>3</v>
       </c>
       <c r="AC7" s="30" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
@@ -2303,15 +2364,15 @@
         <v>4</v>
       </c>
       <c r="AC8" s="30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="2:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E9" s="15">
         <v>0</v>
@@ -2385,7 +2446,7 @@
         <v>5</v>
       </c>
       <c r="AC9" s="30" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="2:29" x14ac:dyDescent="0.3">
@@ -2393,7 +2454,7 @@
         <v>6</v>
       </c>
       <c r="AC10" s="30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="2:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2401,7 +2462,7 @@
         <v>7</v>
       </c>
       <c r="AC11" s="30" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="2:29" x14ac:dyDescent="0.3">
@@ -2477,7 +2538,7 @@
         <v>8</v>
       </c>
       <c r="AC12" s="30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="2:29" x14ac:dyDescent="0.3">
@@ -2521,7 +2582,7 @@
         <v>9</v>
       </c>
       <c r="AC13" s="30" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" spans="2:29" x14ac:dyDescent="0.3">
@@ -2552,7 +2613,7 @@
         <v>10</v>
       </c>
       <c r="AC14" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="2:29" x14ac:dyDescent="0.3">
@@ -2583,7 +2644,7 @@
         <v>11</v>
       </c>
       <c r="AC15" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="2:29" x14ac:dyDescent="0.3">
@@ -2614,7 +2675,7 @@
         <v>12</v>
       </c>
       <c r="AC16" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="5:29" x14ac:dyDescent="0.3">
@@ -2645,7 +2706,7 @@
         <v>13</v>
       </c>
       <c r="AC17" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="5:29" x14ac:dyDescent="0.3">
@@ -2676,7 +2737,7 @@
         <v>14</v>
       </c>
       <c r="AC18" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" spans="5:29" x14ac:dyDescent="0.3">
@@ -2707,7 +2768,7 @@
         <v>15</v>
       </c>
       <c r="AC19" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="5:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>